<commit_message>
Learned services and imperative command, played with the default kubernetes service
</commit_message>
<xml_diff>
--- a/8-Certification_Focused_Learnings/CKA Learning-Checklist.xlsx
+++ b/8-Certification_Focused_Learnings/CKA Learning-Checklist.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\GITHUB-REPO-SLINK\Kubernetes-Certification-Handson\Certification_Focused_Learnings\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\GITHUB-REPO-SLINK\Kubernetes-Certification-Handson\8-Certification_Focused_Learnings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB701C82-0F91-4D7B-8C57-1443380BAE9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D43E8DA-5CBF-48AD-B10F-6BC875EFD305}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="122">
   <si>
     <t>Pod</t>
   </si>
@@ -67,12 +67,6 @@
   </si>
   <si>
     <t>Service</t>
-  </si>
-  <si>
-    <t>Create a Service</t>
-  </si>
-  <si>
-    <t>Expose a Pod</t>
   </si>
   <si>
     <t>Expose a Deployment</t>
@@ -391,6 +385,398 @@
   </si>
   <si>
     <t>There is no imperative command. You have to use the pod manifest to create it.</t>
+  </si>
+  <si>
+    <t>kubectl expose pod nginx --port=80</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Create a Service for the </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>nginx</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Pod and expose port 80. It is a cluster IP service.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">kubectl create service </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>clusterip</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> my-service  --tcp=80:80</t>
+    </r>
+  </si>
+  <si>
+    <t>It creates a clusterip service without any endpoints. 80:80 means &lt;serviceport&gt;:&lt;targetport&gt;</t>
+  </si>
+  <si>
+    <t>Create a nodePort service. Same port mapping as cluster ip but with an additional nodePort field added automatically by the service.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">kubectl create svc </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nodeport</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> my-nodeport-service --tcp=8080:80. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">kubectl create service </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>loadbalancer</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> my-service --tcp=80:80</t>
+    </r>
+  </si>
+  <si>
+    <t>On a cloud Kubernetes cluster, the LoadBalancer can cause an external load balancer to be provisioned.</t>
+  </si>
+  <si>
+    <t>Create NodePort with specific nodePort</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">kubectl create svc </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nodeport</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> my-custom-nodeport --tcp=8080:80 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>--node-port=30005</t>
+    </r>
+  </si>
+  <si>
+    <t>We specify the nodeport thatwe want  using the  --node-port flag</t>
+  </si>
+  <si>
+    <t>Expose a Pod - clusterIP</t>
+  </si>
+  <si>
+    <t>Expose a Pod - nodePort</t>
+  </si>
+  <si>
+    <t>Expose a Pod - loadBalancer</t>
+  </si>
+  <si>
+    <r>
+      <t>kubectl expose pod nginx --port=80</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> --type=LoadBalancer</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>kubectl expose pod nginx</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">--port=80 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>--type=NodePort</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Create a nodePort service for the </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>nginx</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Pod and expose port 80 and map it to nodeport. A random nodeport  port will be assigned</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Create a loadBalancer service for the </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>nginx</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Pod and expose port 80 and map it to nodeport. A random nodeport  port will be assigned. Then finally a cloud load balancer will be create that site infront of the nodePort service to receiv the external traffic.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">kubectl expose deployment my-nginx-deploy </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>--port=80 --type=NodePort</t>
+    </r>
+  </si>
+  <si>
+    <t>Expose a deployment using nodePort service.</t>
+  </si>
+  <si>
+    <t>To add a pod as an endpoint to an already created service</t>
+  </si>
+  <si>
+    <t>1- Find the pod label (kubectl get pods --show-labels), the edit the service (kubectl edit &lt;service name&gt;). Under the selector field, add the pods label. Save the file.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">There is no Imperative command for this use case. Work around is to use </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>patch</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> command.  kubectl patch svc my-service -p '{"spec":{"type":"NodePort"}}'  OR you can use the kubectl </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>edit</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to edit the service on the fly</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve"> kubectl create svc nodeport </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>my-test-svc</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> --tcp=80:80 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">--dry-run=client -o yaml &gt; /tmp/test-svc.yaml . </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Edit the file and apply.</t>
+    </r>
+  </si>
+  <si>
+    <t>Use this option in exams.</t>
+  </si>
+  <si>
+    <t>What happen if you delete the def kubernetes service?</t>
+  </si>
+  <si>
+    <t>In some clusters, it automatically recreaes it. No sure what happen in other. Anyways its is not safe to modify that service.</t>
   </si>
 </sst>
 </file>
@@ -447,7 +833,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -456,8 +842,16 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -740,13 +1134,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:D90"/>
+  <dimension ref="A2:D93"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="44.140625" customWidth="1"/>
+    <col min="1" max="1" width="54" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.42578125" customWidth="1"/>
-    <col min="3" max="3" width="105.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="110.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="133.140625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="228.85546875" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:4" ht="18">
@@ -754,13 +1148,13 @@
         <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="D2" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>67</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -771,13 +1165,13 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>64</v>
-      </c>
-      <c r="C4" t="s">
-        <v>65</v>
-      </c>
-      <c r="D4" t="s">
-        <v>77</v>
+        <v>62</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -785,13 +1179,13 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>64</v>
-      </c>
-      <c r="C5" t="s">
-        <v>70</v>
-      </c>
-      <c r="D5" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>68</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -799,13 +1193,13 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>64</v>
-      </c>
-      <c r="C6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D6" t="s">
-        <v>72</v>
+        <v>62</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -813,13 +1207,13 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>64</v>
-      </c>
-      <c r="C7" t="s">
-        <v>73</v>
-      </c>
-      <c r="D7" t="s">
-        <v>74</v>
+        <v>62</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -827,13 +1221,13 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>64</v>
-      </c>
-      <c r="C8" t="s">
-        <v>75</v>
-      </c>
-      <c r="D8" t="s">
-        <v>76</v>
+        <v>62</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -841,18 +1235,18 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>64</v>
-      </c>
-      <c r="C9" t="s">
+        <v>62</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="D10" s="4" t="s">
         <v>78</v>
-      </c>
-      <c r="D9" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="D10" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="18">
@@ -868,13 +1262,13 @@
         <v>8</v>
       </c>
       <c r="B13" t="s">
-        <v>64</v>
-      </c>
-      <c r="C13" t="s">
-        <v>81</v>
-      </c>
-      <c r="D13" t="s">
-        <v>82</v>
+        <v>62</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -882,13 +1276,13 @@
         <v>9</v>
       </c>
       <c r="B14" t="s">
-        <v>64</v>
-      </c>
-      <c r="C14" t="s">
-        <v>83</v>
-      </c>
-      <c r="D14" t="s">
-        <v>84</v>
+        <v>62</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -896,10 +1290,10 @@
         <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>64</v>
-      </c>
-      <c r="C15" t="s">
-        <v>85</v>
+        <v>62</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -907,10 +1301,10 @@
         <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>64</v>
-      </c>
-      <c r="C16" t="s">
-        <v>86</v>
+        <v>62</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -918,52 +1312,52 @@
         <v>12</v>
       </c>
       <c r="B17" t="s">
-        <v>64</v>
-      </c>
-      <c r="C17" t="s">
-        <v>87</v>
-      </c>
-      <c r="D17" t="s">
-        <v>88</v>
+        <v>62</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="45">
       <c r="A18" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B18" t="s">
+        <v>62</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="45">
+      <c r="A19" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B19" t="s">
+        <v>62</v>
+      </c>
+      <c r="C19" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="B18" t="s">
-        <v>64</v>
-      </c>
-      <c r="C18" t="s">
-        <v>90</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="75">
-      <c r="A19" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="B19" t="s">
-        <v>64</v>
-      </c>
-      <c r="C19" t="s">
-        <v>94</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>95</v>
+      <c r="D19" s="4" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B20" t="s">
-        <v>64</v>
-      </c>
-      <c r="C20" t="s">
-        <v>96</v>
+        <v>62</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="18">
@@ -976,282 +1370,412 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="B23" t="s">
+        <v>62</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="B24" t="s">
+        <v>62</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="2" t="s">
-        <v>16</v>
+        <v>103</v>
+      </c>
+      <c r="B25" t="s">
+        <v>62</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="2" t="s">
         <v>17</v>
       </c>
+      <c r="B26" t="s">
+        <v>62</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="2" t="s">
-        <v>18</v>
+        <v>106</v>
+      </c>
+      <c r="B27" t="s">
+        <v>62</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="2" t="s">
-        <v>19</v>
+        <v>107</v>
+      </c>
+      <c r="B28" t="s">
+        <v>62</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="2" t="s">
-        <v>20</v>
+        <v>108</v>
+      </c>
+      <c r="B29" t="s">
+        <v>62</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="2" t="s">
-        <v>21</v>
+        <v>14</v>
+      </c>
+      <c r="B30" t="s">
+        <v>62</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="2" t="s">
-        <v>22</v>
+        <v>115</v>
+      </c>
+      <c r="B31" t="s">
+        <v>62</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B32" t="s">
+        <v>62</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B33" t="s">
+        <v>62</v>
+      </c>
+      <c r="C33" s="5"/>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B34" t="s">
+        <v>62</v>
+      </c>
+      <c r="C34" s="5"/>
+    </row>
+    <row r="35" spans="1:4">
+      <c r="A35" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B35" t="s">
+        <v>62</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B36" t="s">
+        <v>62</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="18">
+      <c r="A37" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="A38" s="2"/>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="34" spans="1:1" ht="18">
-      <c r="A34" s="1" t="s">
+    <row r="40" spans="1:4">
+      <c r="A40" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="35" spans="1:1">
-      <c r="A35" s="2"/>
-    </row>
-    <row r="36" spans="1:1">
-      <c r="A36" s="2" t="s">
+    <row r="41" spans="1:4">
+      <c r="A41" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="37" spans="1:1">
-      <c r="A37" s="2" t="s">
+    <row r="42" spans="1:4">
+      <c r="A42" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="38" spans="1:1">
-      <c r="A38" s="2" t="s">
+    <row r="44" spans="1:4" ht="18">
+      <c r="A44" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="39" spans="1:1">
-      <c r="A39" s="2" t="s">
+    <row r="45" spans="1:4">
+      <c r="A45" s="2"/>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="A46" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="41" spans="1:1" ht="18">
-      <c r="A41" s="1" t="s">
+    <row r="47" spans="1:4">
+      <c r="A47" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="42" spans="1:1">
-      <c r="A42" s="2"/>
-    </row>
-    <row r="43" spans="1:1">
-      <c r="A43" s="2" t="s">
+    <row r="48" spans="1:4">
+      <c r="A48" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="44" spans="1:1">
-      <c r="A44" s="2" t="s">
+    <row r="50" spans="1:1" ht="18">
+      <c r="A50" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="45" spans="1:1">
-      <c r="A45" s="2" t="s">
+    <row r="51" spans="1:1">
+      <c r="A51" s="2"/>
+    </row>
+    <row r="52" spans="1:1">
+      <c r="A52" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="47" spans="1:1" ht="18">
-      <c r="A47" s="1" t="s">
+    <row r="53" spans="1:1">
+      <c r="A53" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="48" spans="1:1">
-      <c r="A48" s="2"/>
-    </row>
-    <row r="49" spans="1:1">
-      <c r="A49" s="2" t="s">
+    <row r="54" spans="1:1">
+      <c r="A54" s="2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="50" spans="1:1">
-      <c r="A50" s="2" t="s">
+    <row r="56" spans="1:1" ht="18">
+      <c r="A56" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="51" spans="1:1">
-      <c r="A51" s="2" t="s">
+    <row r="57" spans="1:1">
+      <c r="A57" s="2"/>
+    </row>
+    <row r="58" spans="1:1">
+      <c r="A58" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="53" spans="1:1" ht="18">
-      <c r="A53" s="1" t="s">
+    <row r="59" spans="1:1">
+      <c r="A59" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="54" spans="1:1">
-      <c r="A54" s="2"/>
-    </row>
-    <row r="55" spans="1:1">
-      <c r="A55" s="2" t="s">
+    <row r="61" spans="1:1" ht="18">
+      <c r="A61" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="56" spans="1:1">
-      <c r="A56" s="2" t="s">
+    <row r="62" spans="1:1">
+      <c r="A62" s="2"/>
+    </row>
+    <row r="63" spans="1:1">
+      <c r="A63" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="58" spans="1:1" ht="18">
-      <c r="A58" s="1" t="s">
+    <row r="64" spans="1:1">
+      <c r="A64" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="59" spans="1:1">
-      <c r="A59" s="2"/>
-    </row>
-    <row r="60" spans="1:1">
-      <c r="A60" s="2" t="s">
+    <row r="66" spans="1:1" ht="18">
+      <c r="A66" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="61" spans="1:1">
-      <c r="A61" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="63" spans="1:1" ht="18">
-      <c r="A63" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="64" spans="1:1">
-      <c r="A64" s="2"/>
-    </row>
-    <row r="65" spans="1:1">
-      <c r="A65" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="66" spans="1:1">
-      <c r="A66" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
     <row r="67" spans="1:1">
-      <c r="A67" s="2" t="s">
-        <v>46</v>
-      </c>
+      <c r="A67" s="2"/>
     </row>
     <row r="68" spans="1:1">
       <c r="A68" s="2" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="69" spans="1:1">
       <c r="A69" s="2" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="70" spans="1:1">
       <c r="A70" s="2" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
     </row>
     <row r="71" spans="1:1">
       <c r="A71" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="73" spans="1:1" ht="18">
-      <c r="A73" s="1" t="s">
-        <v>51</v>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1">
+      <c r="A72" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1">
+      <c r="A73" s="2" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="74" spans="1:1">
-      <c r="A74" s="2"/>
-    </row>
-    <row r="75" spans="1:1">
-      <c r="A75" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="76" spans="1:1">
-      <c r="A76" s="2" t="s">
-        <v>53</v>
+      <c r="A74" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" ht="18">
+      <c r="A76" s="1" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="77" spans="1:1">
-      <c r="A77" s="2" t="s">
-        <v>54</v>
-      </c>
+      <c r="A77" s="2"/>
     </row>
     <row r="78" spans="1:1">
       <c r="A78" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1">
+      <c r="A79" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1">
+      <c r="A80" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1">
+      <c r="A81" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" ht="18">
+      <c r="A83" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1">
+      <c r="A84" s="2"/>
+    </row>
+    <row r="85" spans="1:1">
+      <c r="A85" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="80" spans="1:1" ht="18">
-      <c r="A80" s="1" t="s">
+    <row r="86" spans="1:1">
+      <c r="A86" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="81" spans="1:1">
-      <c r="A81" s="2"/>
-    </row>
-    <row r="82" spans="1:1">
-      <c r="A82" s="2" t="s">
+    <row r="87" spans="1:1">
+      <c r="A87" s="2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="83" spans="1:1">
-      <c r="A83" s="2" t="s">
+    <row r="89" spans="1:1" ht="18">
+      <c r="A89" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="84" spans="1:1">
-      <c r="A84" s="2" t="s">
+    <row r="90" spans="1:1">
+      <c r="A90" s="2"/>
+    </row>
+    <row r="91" spans="1:1">
+      <c r="A91" s="2" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="86" spans="1:1" ht="18">
-      <c r="A86" s="1" t="s">
+    <row r="92" spans="1:1">
+      <c r="A92" s="2" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="87" spans="1:1">
-      <c r="A87" s="2"/>
-    </row>
-    <row r="88" spans="1:1">
-      <c r="A88" s="2" t="s">
+    <row r="93" spans="1:1">
+      <c r="A93" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="89" spans="1:1">
-      <c r="A89" s="2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="90" spans="1:1">
-      <c r="A90" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C32:C34"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Learned more about imperative commands and services
</commit_message>
<xml_diff>
--- a/8-Certification_Focused_Learnings/CKA Learning-Checklist.xlsx
+++ b/8-Certification_Focused_Learnings/CKA Learning-Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\GITHUB-REPO-SLINK\Kubernetes-Certification-Handson\8-Certification_Focused_Learnings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D43E8DA-5CBF-48AD-B10F-6BC875EFD305}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{259DF2C7-D5C1-4140-A1C6-50BAB9018701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -387,9 +387,6 @@
     <t>There is no imperative command. You have to use the pod manifest to create it.</t>
   </si>
   <si>
-    <t>kubectl expose pod nginx --port=80</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Create a Service for the </t>
     </r>
@@ -777,6 +774,9 @@
   </si>
   <si>
     <t>In some clusters, it automatically recreaes it. No sure what happen in other. Anyways its is not safe to modify that service.</t>
+  </si>
+  <si>
+    <t>kubectl expose pod nginx --port=80. To provide a name to the service : kubectl expose pod nginx --port=80 --target-port=80 --name=web-service</t>
   </si>
 </sst>
 </file>
@@ -845,14 +845,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1150,10 +1150,10 @@
       <c r="B2" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1184,7 +1184,7 @@
       <c r="C5" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="6" t="s">
         <v>66</v>
       </c>
     </row>
@@ -1376,10 +1376,10 @@
         <v>62</v>
       </c>
       <c r="C23" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D23" s="4" t="s">
         <v>97</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -1390,24 +1390,24 @@
         <v>62</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B25" t="s">
+        <v>62</v>
+      </c>
+      <c r="C25" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="B25" t="s">
-        <v>62</v>
-      </c>
-      <c r="C25" s="4" t="s">
+      <c r="D25" s="4" t="s">
         <v>104</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -1418,52 +1418,52 @@
         <v>62</v>
       </c>
       <c r="C26" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D26" s="4" t="s">
         <v>101</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B27" t="s">
         <v>62</v>
       </c>
       <c r="C27" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="D27" s="4" t="s">
         <v>95</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B28" t="s">
         <v>62</v>
       </c>
       <c r="C28" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="D28" s="4" t="s">
         <v>110</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B29" t="s">
+        <v>62</v>
+      </c>
+      <c r="C29" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="B29" t="s">
-        <v>62</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>109</v>
-      </c>
       <c r="D29" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -1474,21 +1474,21 @@
         <v>62</v>
       </c>
       <c r="C30" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="D30" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="D30" s="4" t="s">
+    </row>
+    <row r="31" spans="1:4" ht="30">
+      <c r="A31" s="2" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="31" spans="1:4">
-      <c r="A31" s="2" t="s">
+      <c r="B31" t="s">
+        <v>62</v>
+      </c>
+      <c r="C31" s="4" t="s">
         <v>115</v>
-      </c>
-      <c r="B31" t="s">
-        <v>62</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -1498,8 +1498,8 @@
       <c r="B32" t="s">
         <v>62</v>
       </c>
-      <c r="C32" s="5" t="s">
-        <v>117</v>
+      <c r="C32" s="7" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -1509,7 +1509,7 @@
       <c r="B33" t="s">
         <v>62</v>
       </c>
-      <c r="C33" s="5"/>
+      <c r="C33" s="7"/>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="2" t="s">
@@ -1518,7 +1518,7 @@
       <c r="B34" t="s">
         <v>62</v>
       </c>
-      <c r="C34" s="5"/>
+      <c r="C34" s="7"/>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="2" t="s">
@@ -1528,21 +1528,21 @@
         <v>62</v>
       </c>
       <c r="C35" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D35" s="4" t="s">
         <v>118</v>
-      </c>
-      <c r="D35" s="4" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B36" t="s">
+        <v>62</v>
+      </c>
+      <c r="C36" s="4" t="s">
         <v>120</v>
-      </c>
-      <c r="B36" t="s">
-        <v>62</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="18">

</xml_diff>